<commit_message>
Use the Companies House deficit for cumulative WFM UK losses
The previous commit replaced "more than £240m" with a floor of about
£219m, built from The Grocer's "more than £200m" plus the FY2025 loss.
That moved the figure the wrong way. The Fresh & Wild Ltd accounts
show an accumulated deficit of £224.0m at 31 Dec 2024 and £243.45m at
31 Dec 2025. The report now cites those figures, and the workbook
computes the 2025 deficit from the 2024 balance plus the FY2025 loss.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TAKPMbw4ycQ3qB2SrmkM8Y
</commit_message>
<xml_diff>
--- a/whole-foods-uk-research.xlsx
+++ b/whole-foods-uk-research.xlsx
@@ -50,7 +50,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: The Grocer, 'Whole Foods Market losses in the UK total more than £200m as sales decline', Sept 2025 (FY2024 accounts).</t>
+          <t xml:space="preserve">Source: Fresh &amp; Wild Ltd (company 03576009) FY2024 accounts, Companies House filing history. FY2025 accounts show £243.45m at 31 Dec 2025.</t>
         </r>
       </text>
     </comment>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="680">
   <si>
     <t xml:space="preserve">Whole Foods Market UK — Research Workbook</t>
   </si>
@@ -103,10 +103,10 @@
     <t xml:space="preserve">Financials — down from 35% in FY2023</t>
   </si>
   <si>
-    <t xml:space="preserve">Cumulative pre-tax losses since 2004, floor (£m)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Financials — &gt;£200m through FY2024 plus FY2025 loss</t>
+    <t xml:space="preserve">Accumulated deficit at 31 Dec 2025 (£m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financials — Companies House accounts</t>
   </si>
   <si>
     <t xml:space="preserve">Loss narrowing, FY2022 to FY2025 (£m)</t>
@@ -292,7 +292,7 @@
     <t xml:space="preserve">Cumulative losses</t>
   </si>
   <si>
-    <t xml:space="preserve">CORRECTION: an earlier draft of the report said 'more than £240m'. The source (The Grocer, Sept 2025, FY2024 accounts) says more than £200m through FY2024. Adding the FY2025 loss of £19.4m gives a floor of about £219m. The report has been corrected and Financials!B23 now computes the figure.</t>
+    <t xml:space="preserve">CORRECTION: an earlier version of this workbook gave a floor of £219m, built from the press figure of 'more than £200m'. The Companies House accounts show the actual accumulated deficit: £224.0m at end 2024 and £243.5m at end 2025. Financials!B23 now computes it from the accounts.</t>
   </si>
   <si>
     <t xml:space="preserve">Source access</t>
@@ -454,10 +454,10 @@
     <t xml:space="preserve">Cumulative losses and trajectory</t>
   </si>
   <si>
-    <t xml:space="preserve">Reported cumulative pre-tax losses since 2004, through FY2024 (£m, floor)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Grocer, Sept 2025: 'more than £200m'. A floor, not an exact total.</t>
+    <t xml:space="preserve">Accumulated deficit at 31 Dec 2024 (£m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fresh &amp; Wild Ltd FY2024 accounts, Companies House, balance sheet retained earnings. The press reported it as 'more than £200m'.</t>
   </si>
   <si>
     <t xml:space="preserve">Add: FY2025 pre-tax loss (£m)</t>
@@ -466,10 +466,7 @@
     <t xml:space="preserve">From row 8</t>
   </si>
   <si>
-    <t xml:space="preserve">Implied cumulative losses through FY2025 (£m, floor)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaces the '£240m' in an earlier report draft, which was not supported by the sources</t>
+    <t xml:space="preserve">Ties to the FY2025 accounts figure of £243.45m within rounding. Includes Fresh &amp; Wild losses from before the 2004 acquisition.</t>
   </si>
   <si>
     <t xml:space="preserve">Combined pre-tax losses FY2022–FY2025 (£m)</t>
@@ -2824,9 +2821,9 @@
       <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="5" t="n">
         <f aca="false">Financials!B23</f>
-        <v>219.4</v>
+        <v>243.407</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>15</v>
@@ -3125,231 +3122,231 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>530</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>433</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>531</v>
-      </c>
       <c r="E3" s="3" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>532</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="C4" s="11" t="s">
         <v>533</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="D4" s="4" t="s">
         <v>534</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>535</v>
-      </c>
       <c r="E4" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
+        <v>535</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>536</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="C5" s="11" t="s">
         <v>537</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="D5" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>538</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>535</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>539</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>540</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="C6" s="11" t="s">
         <v>541</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="D6" s="4" t="s">
         <v>542</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>543</v>
-      </c>
       <c r="E6" s="4" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>544</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="C7" s="11" t="s">
         <v>545</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="D7" s="4" t="s">
         <v>546</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>547</v>
-      </c>
       <c r="E7" s="4" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B8" s="11" t="s">
+        <v>547</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>548</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>549</v>
-      </c>
       <c r="D8" s="4" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
+        <v>549</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>550</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="C9" s="11" t="s">
         <v>551</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="D9" s="4" t="s">
         <v>552</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>553</v>
-      </c>
       <c r="E9" s="4" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>554</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>555</v>
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="4" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>557</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="C11" s="11" t="s">
         <v>558</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="D11" s="4" t="s">
         <v>559</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>560</v>
-      </c>
       <c r="E11" s="4" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>561</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="C12" s="11" t="s">
         <v>562</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="D12" s="4" t="s">
         <v>563</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>564</v>
-      </c>
       <c r="E12" s="4" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
+        <v>564</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>565</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="C13" s="11" t="s">
         <v>566</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="D13" s="4" t="s">
         <v>567</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>568</v>
-      </c>
       <c r="E13" s="4" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B14" s="11" t="s">
+        <v>568</v>
+      </c>
+      <c r="C14" s="11" t="s">
         <v>569</v>
       </c>
-      <c r="C14" s="11" t="s">
-        <v>570</v>
-      </c>
       <c r="D14" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="B15" s="11" t="s">
         <v>571</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="C15" s="16" t="s">
         <v>572</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="D15" s="4" t="s">
         <v>573</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>574</v>
-      </c>
       <c r="E15" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
   </sheetData>
@@ -3379,194 +3376,194 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>577</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>578</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>579</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>580</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="11" t="s">
         <v>581</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="D4" s="4" t="s">
         <v>582</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>583</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>584</v>
       </c>
-      <c r="C5" s="11" t="s">
-        <v>585</v>
-      </c>
       <c r="D5" s="4" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="C6" s="11" t="s">
         <v>586</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="D6" s="4" t="s">
         <v>587</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>588</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>589</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="D7" s="4" t="s">
         <v>590</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>591</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>592</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="11" t="s">
         <v>593</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>594</v>
-      </c>
       <c r="D8" s="4" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>594</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>595</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>596</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="C10" s="11" t="s">
         <v>597</v>
       </c>
-      <c r="C10" s="11" t="s">
-        <v>598</v>
-      </c>
       <c r="D10" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>598</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>599</v>
       </c>
-      <c r="C11" s="11" t="s">
-        <v>600</v>
-      </c>
       <c r="D11" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>600</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>601</v>
       </c>
-      <c r="C12" s="11" t="s">
-        <v>602</v>
-      </c>
       <c r="D12" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
+        <v>602</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>603</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="11" t="s">
         <v>604</v>
       </c>
-      <c r="C13" s="11" t="s">
-        <v>605</v>
-      </c>
       <c r="D13" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="C14" s="11" t="s">
         <v>606</v>
       </c>
-      <c r="C14" s="11" t="s">
-        <v>607</v>
-      </c>
       <c r="D14" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="C15" s="11" t="s">
         <v>608</v>
       </c>
-      <c r="C15" s="11" t="s">
-        <v>609</v>
-      </c>
       <c r="D15" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
   </sheetData>
@@ -3604,24 +3601,24 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>611</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>612</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>613</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>614</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3629,16 +3626,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="11" t="s">
+        <v>614</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>615</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="E4" s="33" t="s">
         <v>616</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="E4" s="33" t="s">
-        <v>617</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3646,16 +3643,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="11" t="s">
+        <v>617</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>615</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="E5" s="33" t="s">
         <v>618</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>616</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>379</v>
-      </c>
-      <c r="E5" s="33" t="s">
-        <v>619</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3663,16 +3660,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="11" t="s">
+        <v>619</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>615</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="E6" s="33" t="s">
         <v>620</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>616</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="E6" s="33" t="s">
-        <v>621</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3680,16 +3677,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="11" t="s">
+        <v>621</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>615</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E7" s="33" t="s">
         <v>622</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>616</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="E7" s="33" t="s">
-        <v>623</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3697,16 +3694,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="11" t="s">
+        <v>623</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>624</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="E8" s="33" t="s">
         <v>625</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="E8" s="33" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3714,16 +3711,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="11" t="s">
+        <v>626</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="E9" s="33" t="s">
         <v>627</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>369</v>
-      </c>
-      <c r="E9" s="33" t="s">
-        <v>628</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3731,16 +3728,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="11" t="s">
+        <v>628</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>629</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="E10" s="33" t="s">
         <v>630</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>379</v>
-      </c>
-      <c r="E10" s="33" t="s">
-        <v>631</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3748,16 +3745,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="11" t="s">
+        <v>631</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>632</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="E11" s="33" t="s">
         <v>633</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="E11" s="33" t="s">
-        <v>634</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3765,16 +3762,16 @@
         <v>9</v>
       </c>
       <c r="B12" s="11" t="s">
+        <v>634</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>635</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="E12" s="33" t="s">
         <v>636</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="E12" s="33" t="s">
-        <v>637</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3782,16 +3779,16 @@
         <v>10</v>
       </c>
       <c r="B13" s="11" t="s">
+        <v>637</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>638</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E13" s="33" t="s">
         <v>639</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="E13" s="33" t="s">
-        <v>640</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3799,16 +3796,16 @@
         <v>11</v>
       </c>
       <c r="B14" s="11" t="s">
+        <v>640</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>615</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E14" s="33" t="s">
         <v>641</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>616</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="E14" s="33" t="s">
-        <v>642</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3816,16 +3813,16 @@
         <v>12</v>
       </c>
       <c r="B15" s="11" t="s">
+        <v>642</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>643</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="4" t="s">
         <v>644</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="E15" s="33" t="s">
         <v>645</v>
-      </c>
-      <c r="E15" s="33" t="s">
-        <v>646</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3833,16 +3830,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="11" t="s">
+        <v>646</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>644</v>
+      </c>
+      <c r="E16" s="33" t="s">
         <v>647</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>504</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>645</v>
-      </c>
-      <c r="E16" s="33" t="s">
-        <v>648</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3850,16 +3847,16 @@
         <v>14</v>
       </c>
       <c r="B17" s="11" t="s">
+        <v>648</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>649</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="4" t="s">
+        <v>644</v>
+      </c>
+      <c r="E17" s="33" t="s">
         <v>650</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>645</v>
-      </c>
-      <c r="E17" s="33" t="s">
-        <v>651</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3867,16 +3864,16 @@
         <v>15</v>
       </c>
       <c r="B18" s="11" t="s">
+        <v>651</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>652</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="E18" s="33" t="s">
         <v>653</v>
-      </c>
-      <c r="E18" s="33" t="s">
-        <v>654</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3884,16 +3881,16 @@
         <v>16</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C19" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>655</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="E19" s="33" t="s">
         <v>656</v>
-      </c>
-      <c r="E19" s="33" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3901,16 +3898,16 @@
         <v>17</v>
       </c>
       <c r="B20" s="11" t="s">
+        <v>657</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>658</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="D20" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E20" s="33" t="s">
         <v>659</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="E20" s="33" t="s">
-        <v>660</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3918,16 +3915,16 @@
         <v>18</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="E21" s="33" t="s">
         <v>661</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>312</v>
-      </c>
-      <c r="E21" s="33" t="s">
-        <v>662</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3935,16 +3932,16 @@
         <v>19</v>
       </c>
       <c r="B22" s="11" t="s">
+        <v>662</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>663</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="D22" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E22" s="33" t="s">
         <v>664</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="E22" s="33" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3952,16 +3949,16 @@
         <v>20</v>
       </c>
       <c r="B23" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>666</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="D23" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E23" s="33" t="s">
         <v>667</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>359</v>
-      </c>
-      <c r="E23" s="33" t="s">
-        <v>668</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3969,14 +3966,14 @@
         <v>21</v>
       </c>
       <c r="B24" s="11" t="s">
+        <v>668</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>669</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>670</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="33" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3984,16 +3981,16 @@
         <v>22</v>
       </c>
       <c r="B25" s="11" t="s">
+        <v>671</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>672</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="D25" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E25" s="33" t="s">
         <v>673</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="E25" s="33" t="s">
-        <v>674</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4001,16 +3998,16 @@
         <v>23</v>
       </c>
       <c r="B26" s="11" t="s">
+        <v>674</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>675</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>496</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="E26" s="33" t="s">
         <v>676</v>
-      </c>
-      <c r="E26" s="33" t="s">
-        <v>677</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4018,14 +4015,14 @@
         <v>24</v>
       </c>
       <c r="B27" s="11" t="s">
+        <v>677</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>678</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>679</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="33" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
   </sheetData>
@@ -4567,8 +4564,8 @@
       <c r="A21" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="B21" s="21" t="n">
-        <v>200</v>
+      <c r="B21" s="17" t="n">
+        <v>224.007</v>
       </c>
       <c r="G21" s="11" t="s">
         <v>132</v>
@@ -4588,19 +4585,19 @@
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" s="20" t="n">
+        <f aca="false">B21+B22</f>
+        <v>243.407</v>
+      </c>
+      <c r="G23" s="16" t="s">
         <v>135</v>
-      </c>
-      <c r="B23" s="23" t="n">
-        <f aca="false">B21+B22</f>
-        <v>219.4</v>
-      </c>
-      <c r="G23" s="16" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B24" s="20" t="n">
         <f aca="false">SUM(C8:F8)</f>
@@ -4624,14 +4621,14 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B26" s="20" t="n">
         <f aca="false">B25/3</f>
         <v>2.3</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4643,7 +4640,7 @@
         <v>8.43478260869565</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -4682,79 +4679,79 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>152</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="C4" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>156</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>157</v>
       </c>
       <c r="E4" s="21" t="n">
         <v>80000</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="I4" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="K4" s="4" t="s">
         <v>161</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>162</v>
       </c>
       <c r="L4" s="23" t="n">
         <f aca="false">COUNTIF(H4:H15,"Open")</f>
@@ -4763,31 +4760,31 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="C5" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="I5" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="G5" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="I5" s="11" t="s">
+      <c r="K5" s="4" t="s">
         <v>167</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>168</v>
       </c>
       <c r="L5" s="23" t="n">
         <f aca="false">COUNTIF(D4:D15,"Daily Shop")</f>
@@ -4796,28 +4793,28 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="C6" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="K6" s="4" t="s">
         <v>170</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>171</v>
       </c>
       <c r="L6" s="23" t="n">
         <f aca="false">COUNTIF(G4:G15,"Yes")</f>
@@ -4826,28 +4823,28 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>172</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="C7" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="K7" s="4" t="s">
         <v>174</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>175</v>
       </c>
       <c r="L7" s="23" t="n">
         <f aca="false">COUNTIF(F4:F15,"&gt;="&amp;DATE(2026,1,1))</f>
@@ -4856,28 +4853,28 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>176</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="C8" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="K8" s="4" t="s">
         <v>178</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>179</v>
       </c>
       <c r="L8" s="23" t="n">
         <f aca="false">COUNTIF(C20:C22,"Store")</f>
@@ -4886,16 +4883,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="C9" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>182</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>183</v>
       </c>
       <c r="E9" s="21" t="n">
         <v>21800</v>
@@ -4904,16 +4901,16 @@
         <v>45741</v>
       </c>
       <c r="G9" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>160</v>
-      </c>
       <c r="I9" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="K9" s="4" t="s">
         <v>184</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>185</v>
       </c>
       <c r="L9" s="6" t="n">
         <f aca="false">IFERROR(L4/Financials!F17-1,"")</f>
@@ -4922,232 +4919,232 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>186</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="C10" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>188</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>189</v>
       </c>
       <c r="F10" s="24" t="n">
         <v>46114</v>
       </c>
       <c r="G10" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="I10" s="11" t="s">
         <v>190</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="I10" s="11" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="C11" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>194</v>
-      </c>
       <c r="D11" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F11" s="24" t="n">
         <v>46135</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="C12" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>198</v>
-      </c>
       <c r="D12" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>46156</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="C13" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>201</v>
-      </c>
       <c r="D13" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F13" s="24" t="n">
         <v>46170</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B14" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>203</v>
-      </c>
       <c r="C14" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F14" s="24" t="n">
         <v>46177</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B15" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="C15" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>206</v>
-      </c>
       <c r="D15" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F15" s="24" t="n">
         <v>46184</v>
       </c>
       <c r="G15" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="H15" s="4" t="s">
-        <v>160</v>
-      </c>
       <c r="I15" s="11" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="25" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>213</v>
-      </c>
       <c r="E19" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>215</v>
-      </c>
       <c r="C20" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D20" s="24" t="n">
         <v>45453</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>218</v>
-      </c>
       <c r="C21" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D21" s="24" t="n">
         <v>45453</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="C22" s="4" t="s">
         <v>221</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>222</v>
       </c>
       <c r="D22" s="24" t="n">
         <v>45453</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="16" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B23" s="16"/>
       <c r="C23" s="16"/>
@@ -5192,234 +5189,234 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>232</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B4" s="18" t="n">
         <v>0.273</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>234</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="E4" s="11" t="s">
         <v>235</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="F4" s="11" t="s">
         <v>236</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B5" s="18" t="n">
         <v>0.155</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="D5" s="11" t="s">
         <v>239</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="E5" s="11" t="s">
         <v>240</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="F5" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="G5" s="11" t="s">
         <v>241</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>237</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>0.101</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="D6" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="E6" s="11" t="s">
         <v>245</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>246</v>
-      </c>
       <c r="F6" s="11" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B7" s="18" t="n">
         <v>0.077</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="D7" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="D7" s="11" t="s">
-        <v>245</v>
-      </c>
       <c r="E7" s="11" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>0.045</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="D8" s="11" t="s">
         <v>250</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="E8" s="11" t="s">
         <v>251</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="F8" s="11" t="s">
         <v>252</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="G8" s="11" t="s">
         <v>253</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B9" s="18" t="n">
         <v>0.045</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D9" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="E9" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="F9" s="11" t="s">
         <v>257</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="G9" s="11" t="s">
         <v>258</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="11" t="s">
         <v>261</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="E10" s="11" t="s">
         <v>262</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="F10" s="11" t="s">
         <v>263</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="G10" s="11" t="s">
         <v>264</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>266</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="D11" s="11" t="s">
+      <c r="E11" s="11" t="s">
         <v>267</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="F11" s="11" t="s">
         <v>268</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="G11" s="11" t="s">
         <v>269</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="11" t="s">
         <v>272</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="E12" s="11" t="s">
         <v>273</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="F12" s="11" t="s">
         <v>274</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="G12" s="11" t="s">
         <v>275</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B15" s="19" t="n">
         <f aca="false">B6+B7</f>
@@ -5428,7 +5425,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B16" s="19" t="n">
         <f aca="false">B8+B9</f>
@@ -5437,12 +5434,12 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B19" s="26" t="n">
         <v>129.83</v>
@@ -5450,7 +5447,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B20" s="26" t="n">
         <v>100.29</v>
@@ -5458,19 +5455,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B21" s="19" t="n">
         <f aca="false">IFERROR(B19/B20-1,"")</f>
         <v>0.294545817130322</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B22" s="27" t="n">
         <f aca="false">B19-B20</f>
@@ -5479,26 +5476,26 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>288</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B26" s="17" t="n">
         <v>-10.3</v>
@@ -5513,7 +5510,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B27" s="17" t="n">
         <v>53</v>
@@ -5528,7 +5525,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B28" s="17" t="n">
         <v>48.8</v>
@@ -5543,12 +5540,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="25" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5561,7 +5558,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B33" s="17" t="n">
         <v>1.3</v>
@@ -5569,7 +5566,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B34" s="19" t="n">
         <f aca="false">IFERROR(B33/B32,"")</f>
@@ -5578,7 +5575,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B35" s="6" t="n">
         <f aca="false">IFERROR(B32/Financials!F5,"")</f>
@@ -5587,12 +5584,12 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B38" s="21" t="n">
         <v>35</v>
@@ -5600,7 +5597,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B39" s="21" t="n">
         <v>37</v>
@@ -5608,7 +5605,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B40" s="23" t="n">
         <f aca="false">B38-B39</f>
@@ -5617,7 +5614,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="25" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
   </sheetData>
@@ -5648,45 +5645,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>305</v>
-      </c>
       <c r="E3" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B4" s="22" t="n">
         <v>1.86</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B5" s="22" t="n">
         <v>3.2</v>
@@ -5699,12 +5696,12 @@
         <v>3.13725490196078</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B6" s="22" t="n">
         <v>3.7</v>
@@ -5717,12 +5714,12 @@
         <v>3.44827586206897</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B7" s="22" t="n">
         <v>3.9</v>
@@ -5735,43 +5732,43 @@
         <v>3.74280230326296</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">B6/B4-1</f>
         <v>0.989247311827957</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>319</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B12" s="22" t="n">
         <v>2.43</v>
@@ -5786,7 +5783,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B13" s="22" t="n">
         <v>0.5176</v>
@@ -5801,7 +5798,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B14" s="22" t="n">
         <v>0.5409</v>
@@ -5816,7 +5813,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B15" s="22" t="n">
         <v>0.2082</v>
@@ -5831,7 +5828,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B16" s="29" t="n">
         <f aca="false">SUM(B12:B15)</f>
@@ -5844,31 +5841,31 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B17" s="30" t="n">
         <f aca="false">B16-B6</f>
         <v>-0.00329999999999986</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B20" s="6" t="n">
         <f aca="false">IFERROR(Financials!E5/(B6*1000),"")</f>
         <v>0.0233513513513514</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -5897,45 +5894,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>334</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
+        <v>335</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>336</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="C4" s="4" t="s">
         <v>337</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5943,10 +5940,10 @@
         <v>42902</v>
       </c>
       <c r="B6" s="11" t="s">
+        <v>339</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>340</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5954,21 +5951,21 @@
         <v>42975</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
+        <v>342</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>343</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="C8" s="4" t="s">
         <v>344</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5976,10 +5973,10 @@
         <v>44454</v>
       </c>
       <c r="B9" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>346</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5987,10 +5984,10 @@
         <v>101</v>
       </c>
       <c r="B10" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>348</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5998,29 +5995,29 @@
         <v>45140</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="31" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B12" s="11" t="s">
+        <v>350</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>351</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="31" t="s">
+        <v>352</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>353</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>354</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>50</v>
@@ -6028,13 +6025,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="31" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6042,18 +6039,18 @@
         <v>45453</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="31" t="s">
+        <v>356</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>357</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>358</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>54</v>
@@ -6061,24 +6058,24 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="31" t="s">
+        <v>358</v>
+      </c>
+      <c r="B17" s="11" t="s">
         <v>359</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>360</v>
-      </c>
       <c r="C17" s="4" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="31" t="s">
+        <v>360</v>
+      </c>
+      <c r="B18" s="11" t="s">
         <v>361</v>
       </c>
-      <c r="B18" s="11" t="s">
-        <v>362</v>
-      </c>
       <c r="C18" s="4" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6086,32 +6083,32 @@
         <v>45741</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="31" t="s">
+        <v>363</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>364</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>365</v>
-      </c>
       <c r="C20" s="4" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
+        <v>365</v>
+      </c>
+      <c r="B21" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="B21" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="C21" s="4" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6119,21 +6116,21 @@
         <v>45923</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="31" t="s">
+        <v>368</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>369</v>
       </c>
-      <c r="B23" s="11" t="s">
-        <v>370</v>
-      </c>
       <c r="C23" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6141,10 +6138,10 @@
         <v>46114</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6152,10 +6149,10 @@
         <v>46135</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6163,10 +6160,10 @@
         <v>46156</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6174,10 +6171,10 @@
         <v>46170</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6185,10 +6182,10 @@
         <v>46177</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6196,43 +6193,43 @@
         <v>46184</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="31" t="s">
+        <v>376</v>
+      </c>
+      <c r="B30" s="11" t="s">
         <v>377</v>
       </c>
-      <c r="B30" s="11" t="s">
-        <v>378</v>
-      </c>
       <c r="C30" s="4" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="31" t="s">
+        <v>378</v>
+      </c>
+      <c r="B31" s="11" t="s">
         <v>379</v>
       </c>
-      <c r="B31" s="11" t="s">
-        <v>380</v>
-      </c>
       <c r="C31" s="4" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="31" t="s">
+        <v>380</v>
+      </c>
+      <c r="B32" s="11" t="s">
         <v>381</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="C32" s="4" t="s">
         <v>382</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>383</v>
       </c>
     </row>
   </sheetData>
@@ -6262,196 +6259,196 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>386</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>387</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="B4" s="16" t="s">
         <v>389</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="C4" s="11" t="s">
         <v>390</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>392</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="C5" s="11" t="s">
         <v>393</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>395</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="C6" s="11" t="s">
         <v>396</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>398</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="C7" s="11" t="s">
         <v>399</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>401</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="C8" s="11" t="s">
         <v>402</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>404</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="C9" s="11" t="s">
         <v>405</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>407</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="C10" s="11" t="s">
         <v>408</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>410</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="C11" s="11" t="s">
         <v>411</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B29" s="23" t="n">
         <f aca="false">COUNTA(A14:A28)</f>
@@ -6460,7 +6457,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B30" s="21" t="n">
         <v>141</v>
@@ -6468,167 +6465,167 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>432</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>335</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>434</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="C34" s="11" t="s">
         <v>435</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>436</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>437</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>438</v>
       </c>
       <c r="C35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="C36" s="11" t="s">
         <v>439</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="C36" s="11" t="s">
-        <v>440</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="B37" s="4" t="s">
         <v>441</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>442</v>
       </c>
       <c r="C37" s="11"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>443</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="C38" s="11" t="s">
         <v>444</v>
-      </c>
-      <c r="C38" s="11" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="C39" s="11" t="s">
         <v>446</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C39" s="11" t="s">
-        <v>447</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>448</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="C40" s="11" t="s">
         <v>449</v>
-      </c>
-      <c r="C40" s="11" t="s">
-        <v>450</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="B41" s="4" t="s">
         <v>451</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="C41" s="11" t="s">
         <v>452</v>
-      </c>
-      <c r="C41" s="11" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B42" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="C42" s="11" t="s">
         <v>452</v>
-      </c>
-      <c r="C42" s="11" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="B43" s="4" t="s">
         <v>455</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="C43" s="11" t="s">
         <v>456</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>458</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>459</v>
-      </c>
       <c r="C44" s="11" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="B45" s="4" t="s">
         <v>460</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="C45" s="11" t="s">
         <v>461</v>
-      </c>
-      <c r="C45" s="11" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="9" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B48" s="21" t="n">
         <v>500</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B49" s="21" t="n">
         <v>17</v>
@@ -6636,19 +6633,19 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B50" s="19" t="n">
         <f aca="false">IFERROR(B49/B48,"")</f>
         <v>0.034</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B51" s="21" t="n">
         <v>50</v>
@@ -6682,278 +6679,278 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>473</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>474</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>475</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B4" s="18" t="n">
         <v>1.33</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>477</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="E4" s="11" t="s">
         <v>478</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B5" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="D5" s="11" t="s">
         <v>477</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>478</v>
       </c>
       <c r="E5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>0.64</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="D6" s="11" t="s">
         <v>477</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>478</v>
       </c>
       <c r="E6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B7" s="18" t="n">
         <v>0.68</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="D7" s="11" t="s">
         <v>477</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>478</v>
       </c>
       <c r="E7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>0.33</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D8" s="11" t="s">
+        <v>483</v>
+      </c>
+      <c r="E8" s="11" t="s">
         <v>484</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
+        <v>485</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>486</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="C9" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>487</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>388</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>488</v>
       </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B10" s="21" t="n">
         <v>15</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D10" s="11" t="s">
+        <v>489</v>
+      </c>
+      <c r="E10" s="11" t="s">
         <v>490</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B11" s="18" t="n">
         <v>0.45</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D11" s="11" t="s">
+        <v>492</v>
+      </c>
+      <c r="E11" s="11" t="s">
         <v>493</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B12" s="18" t="n">
         <v>0.32</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D12" s="11" t="s">
+        <v>495</v>
+      </c>
+      <c r="E12" s="11" t="s">
         <v>496</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B13" s="18" t="n">
         <v>0.73</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>499</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>500</v>
       </c>
       <c r="E13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B14" s="18" t="n">
         <v>0.69</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="E14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B15" s="18" t="n">
         <v>0.42</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="D15" s="11" t="s">
+        <v>503</v>
+      </c>
+      <c r="E15" s="11" t="s">
         <v>504</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>505</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B16" s="18" t="n">
         <v>0.83</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="E16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B17" s="18" t="n">
         <v>0.24</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="E17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B18" s="18" t="n">
         <v>0.33</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="E18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B19" s="19" t="n">
         <f aca="false">B18-B17</f>
         <v>0.09</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>111</v>
@@ -6962,127 +6959,127 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B20" s="18" t="n">
         <v>0.75</v>
       </c>
       <c r="C20" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="D20" s="11" t="s">
         <v>512</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="E20" s="11" t="s">
         <v>513</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B21" s="18" t="n">
         <v>0.46</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>512</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="E21" s="11" t="s">
         <v>513</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B22" s="18" t="n">
         <v>0.27</v>
       </c>
       <c r="C22" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="D22" s="11" t="s">
         <v>512</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>513</v>
       </c>
       <c r="E22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B23" s="18" t="n">
         <v>0.7</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="D23" s="11" t="s">
         <v>518</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>519</v>
       </c>
       <c r="E23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B24" s="18" t="n">
         <v>0.55</v>
       </c>
       <c r="C24" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>518</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>519</v>
       </c>
       <c r="E24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B25" s="18" t="n">
         <v>0.7</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>518</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>519</v>
       </c>
       <c r="E25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B26" s="18" t="n">
         <v>0.92</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D26" s="11" t="s">
+        <v>522</v>
+      </c>
+      <c r="E26" s="16" t="s">
         <v>523</v>
-      </c>
-      <c r="E26" s="16" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
+        <v>524</v>
+      </c>
+      <c r="B27" s="11" t="s">
         <v>525</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="C27" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="D27" s="11" t="s">
         <v>526</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>387</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>527</v>
       </c>
       <c r="E27" s="11"/>
     </row>

</xml_diff>